<commit_message>
Actualizar formato Visita 2 GFPI-F023.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Formatos/Visita 2 GFPI-F023.xlsx
+++ b/Formatos/Visita 2 GFPI-F023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SEANT\OneDrive\Documents\Seto 2026\sena\Manual SENA Etapa Productiva\manual-aprendiz-sena\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0630D33E-B5D0-4F12-A43A-9112395366C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FB8EBA-F1E6-4458-A15B-89CCBCFED77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BC3553EE-4E49-4F2A-B03E-CFAC4EB3009B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1293,18 +1293,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1313,6 +1301,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1494,7 +1494,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1508,7 +1508,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="8" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2102,15 +2102,15 @@
       </c>
       <c r="C14" s="107"/>
       <c r="D14" s="97"/>
-      <c r="E14" s="119"/>
-      <c r="F14" s="120"/>
-      <c r="G14" s="120"/>
-      <c r="H14" s="120"/>
-      <c r="I14" s="120"/>
-      <c r="J14" s="120"/>
-      <c r="K14" s="120"/>
-      <c r="L14" s="120"/>
-      <c r="M14" s="121"/>
+      <c r="E14" s="122"/>
+      <c r="F14" s="123"/>
+      <c r="G14" s="123"/>
+      <c r="H14" s="123"/>
+      <c r="I14" s="123"/>
+      <c r="J14" s="123"/>
+      <c r="K14" s="123"/>
+      <c r="L14" s="123"/>
+      <c r="M14" s="124"/>
     </row>
     <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="105"/>
@@ -2136,15 +2136,15 @@
       </c>
       <c r="C16" s="107"/>
       <c r="D16" s="97"/>
-      <c r="E16" s="119"/>
-      <c r="F16" s="120"/>
-      <c r="G16" s="120"/>
-      <c r="H16" s="120"/>
-      <c r="I16" s="120"/>
-      <c r="J16" s="120"/>
-      <c r="K16" s="120"/>
-      <c r="L16" s="120"/>
-      <c r="M16" s="121"/>
+      <c r="E16" s="122"/>
+      <c r="F16" s="123"/>
+      <c r="G16" s="123"/>
+      <c r="H16" s="123"/>
+      <c r="I16" s="123"/>
+      <c r="J16" s="123"/>
+      <c r="K16" s="123"/>
+      <c r="L16" s="123"/>
+      <c r="M16" s="124"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="105"/>
@@ -2153,15 +2153,15 @@
       </c>
       <c r="C17" s="107"/>
       <c r="D17" s="97"/>
-      <c r="E17" s="119"/>
-      <c r="F17" s="120"/>
-      <c r="G17" s="120"/>
-      <c r="H17" s="120"/>
-      <c r="I17" s="120"/>
-      <c r="J17" s="120"/>
-      <c r="K17" s="120"/>
-      <c r="L17" s="120"/>
-      <c r="M17" s="121"/>
+      <c r="E17" s="122"/>
+      <c r="F17" s="123"/>
+      <c r="G17" s="123"/>
+      <c r="H17" s="123"/>
+      <c r="I17" s="123"/>
+      <c r="J17" s="123"/>
+      <c r="K17" s="123"/>
+      <c r="L17" s="123"/>
+      <c r="M17" s="124"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="105"/>
@@ -2170,15 +2170,15 @@
       </c>
       <c r="C18" s="107"/>
       <c r="D18" s="97"/>
-      <c r="E18" s="119"/>
-      <c r="F18" s="120"/>
-      <c r="G18" s="120"/>
-      <c r="H18" s="120"/>
-      <c r="I18" s="120"/>
-      <c r="J18" s="120"/>
-      <c r="K18" s="120"/>
-      <c r="L18" s="120"/>
-      <c r="M18" s="121"/>
+      <c r="E18" s="122"/>
+      <c r="F18" s="123"/>
+      <c r="G18" s="123"/>
+      <c r="H18" s="123"/>
+      <c r="I18" s="123"/>
+      <c r="J18" s="123"/>
+      <c r="K18" s="123"/>
+      <c r="L18" s="123"/>
+      <c r="M18" s="124"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="105"/>
@@ -2187,15 +2187,15 @@
       </c>
       <c r="C19" s="107"/>
       <c r="D19" s="97"/>
-      <c r="E19" s="119"/>
-      <c r="F19" s="120"/>
-      <c r="G19" s="120"/>
-      <c r="H19" s="120"/>
-      <c r="I19" s="120"/>
-      <c r="J19" s="120"/>
-      <c r="K19" s="120"/>
-      <c r="L19" s="120"/>
-      <c r="M19" s="121"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="123"/>
+      <c r="G19" s="123"/>
+      <c r="H19" s="123"/>
+      <c r="I19" s="123"/>
+      <c r="J19" s="123"/>
+      <c r="K19" s="123"/>
+      <c r="L19" s="123"/>
+      <c r="M19" s="124"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="105"/>
@@ -2314,15 +2314,15 @@
       </c>
       <c r="C26" s="107"/>
       <c r="D26" s="97"/>
-      <c r="E26" s="119"/>
-      <c r="F26" s="120"/>
-      <c r="G26" s="120"/>
-      <c r="H26" s="120"/>
-      <c r="I26" s="120"/>
-      <c r="J26" s="120"/>
-      <c r="K26" s="120"/>
-      <c r="L26" s="120"/>
-      <c r="M26" s="121"/>
+      <c r="E26" s="122"/>
+      <c r="F26" s="123"/>
+      <c r="G26" s="123"/>
+      <c r="H26" s="123"/>
+      <c r="I26" s="123"/>
+      <c r="J26" s="123"/>
+      <c r="K26" s="123"/>
+      <c r="L26" s="123"/>
+      <c r="M26" s="124"/>
     </row>
     <row r="27" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
@@ -2333,15 +2333,15 @@
       </c>
       <c r="C27" s="107"/>
       <c r="D27" s="97"/>
-      <c r="E27" s="119"/>
-      <c r="F27" s="120"/>
-      <c r="G27" s="120"/>
-      <c r="H27" s="120"/>
-      <c r="I27" s="120"/>
-      <c r="J27" s="120"/>
-      <c r="K27" s="120"/>
-      <c r="L27" s="120"/>
-      <c r="M27" s="121"/>
+      <c r="E27" s="122"/>
+      <c r="F27" s="123"/>
+      <c r="G27" s="123"/>
+      <c r="H27" s="123"/>
+      <c r="I27" s="123"/>
+      <c r="J27" s="123"/>
+      <c r="K27" s="123"/>
+      <c r="L27" s="123"/>
+      <c r="M27" s="124"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
@@ -2350,15 +2350,15 @@
       </c>
       <c r="C28" s="107"/>
       <c r="D28" s="97"/>
-      <c r="E28" s="119"/>
-      <c r="F28" s="120"/>
-      <c r="G28" s="120"/>
-      <c r="H28" s="120"/>
-      <c r="I28" s="120"/>
-      <c r="J28" s="120"/>
-      <c r="K28" s="120"/>
-      <c r="L28" s="120"/>
-      <c r="M28" s="121"/>
+      <c r="E28" s="122"/>
+      <c r="F28" s="123"/>
+      <c r="G28" s="123"/>
+      <c r="H28" s="123"/>
+      <c r="I28" s="123"/>
+      <c r="J28" s="123"/>
+      <c r="K28" s="123"/>
+      <c r="L28" s="123"/>
+      <c r="M28" s="124"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
@@ -2367,15 +2367,15 @@
       </c>
       <c r="C29" s="107"/>
       <c r="D29" s="97"/>
-      <c r="E29" s="119"/>
-      <c r="F29" s="120"/>
-      <c r="G29" s="120"/>
-      <c r="H29" s="120"/>
-      <c r="I29" s="120"/>
-      <c r="J29" s="120"/>
-      <c r="K29" s="120"/>
-      <c r="L29" s="120"/>
-      <c r="M29" s="121"/>
+      <c r="E29" s="122"/>
+      <c r="F29" s="123"/>
+      <c r="G29" s="123"/>
+      <c r="H29" s="123"/>
+      <c r="I29" s="123"/>
+      <c r="J29" s="123"/>
+      <c r="K29" s="123"/>
+      <c r="L29" s="123"/>
+      <c r="M29" s="124"/>
     </row>
     <row r="30" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
@@ -2386,15 +2386,15 @@
       </c>
       <c r="C30" s="107"/>
       <c r="D30" s="97"/>
-      <c r="E30" s="119"/>
-      <c r="F30" s="120"/>
-      <c r="G30" s="120"/>
-      <c r="H30" s="120"/>
-      <c r="I30" s="120"/>
-      <c r="J30" s="120"/>
-      <c r="K30" s="120"/>
-      <c r="L30" s="120"/>
-      <c r="M30" s="121"/>
+      <c r="E30" s="122"/>
+      <c r="F30" s="123"/>
+      <c r="G30" s="123"/>
+      <c r="H30" s="123"/>
+      <c r="I30" s="123"/>
+      <c r="J30" s="123"/>
+      <c r="K30" s="123"/>
+      <c r="L30" s="123"/>
+      <c r="M30" s="124"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
@@ -2403,15 +2403,15 @@
       </c>
       <c r="C31" s="107"/>
       <c r="D31" s="97"/>
-      <c r="E31" s="119"/>
-      <c r="F31" s="120"/>
-      <c r="G31" s="120"/>
-      <c r="H31" s="120"/>
-      <c r="I31" s="120"/>
-      <c r="J31" s="120"/>
-      <c r="K31" s="120"/>
-      <c r="L31" s="120"/>
-      <c r="M31" s="121"/>
+      <c r="E31" s="122"/>
+      <c r="F31" s="123"/>
+      <c r="G31" s="123"/>
+      <c r="H31" s="123"/>
+      <c r="I31" s="123"/>
+      <c r="J31" s="123"/>
+      <c r="K31" s="123"/>
+      <c r="L31" s="123"/>
+      <c r="M31" s="124"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
@@ -2437,23 +2437,23 @@
       </c>
       <c r="C33" s="107"/>
       <c r="D33" s="97"/>
-      <c r="E33" s="119"/>
-      <c r="F33" s="120"/>
-      <c r="G33" s="120"/>
-      <c r="H33" s="120"/>
-      <c r="I33" s="120"/>
-      <c r="J33" s="120"/>
-      <c r="K33" s="120"/>
-      <c r="L33" s="120"/>
-      <c r="M33" s="121"/>
+      <c r="E33" s="122"/>
+      <c r="F33" s="123"/>
+      <c r="G33" s="123"/>
+      <c r="H33" s="123"/>
+      <c r="I33" s="123"/>
+      <c r="J33" s="123"/>
+      <c r="K33" s="123"/>
+      <c r="L33" s="123"/>
+      <c r="M33" s="124"/>
     </row>
     <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7"/>
-      <c r="B34" s="122" t="s">
+      <c r="B34" s="119" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="123"/>
-      <c r="D34" s="124"/>
+      <c r="C34" s="120"/>
+      <c r="D34" s="121"/>
       <c r="E34" s="116"/>
       <c r="F34" s="117"/>
       <c r="G34" s="117"/>
@@ -2628,11 +2628,11 @@
       <c r="D44" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E44" s="122" t="s">
+      <c r="E44" s="119" t="s">
         <v>48</v>
       </c>
-      <c r="F44" s="123"/>
-      <c r="G44" s="123"/>
+      <c r="F44" s="120"/>
+      <c r="G44" s="120"/>
       <c r="H44" s="116"/>
       <c r="I44" s="117"/>
       <c r="J44" s="118"/>
@@ -2739,6 +2739,8 @@
       <c r="C50" s="33"/>
       <c r="D50" s="34"/>
       <c r="E50" s="35"/>
+      <c r="F50" s="34"/>
+      <c r="G50" s="35"/>
       <c r="H50" s="41"/>
       <c r="I50" s="42"/>
       <c r="J50" s="43"/>
@@ -3201,7 +3203,8 @@
     </row>
     <row r="81" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="166">
+    <mergeCell ref="F50:G50"/>
     <mergeCell ref="F80:G80"/>
     <mergeCell ref="A38:M40"/>
     <mergeCell ref="C79:J79"/>
@@ -3225,6 +3228,7 @@
     <mergeCell ref="I72:J76"/>
     <mergeCell ref="K72:M76"/>
     <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B36:D36"/>
     <mergeCell ref="C9:M9"/>
     <mergeCell ref="A8:M8"/>
     <mergeCell ref="E14:M14"/>
@@ -3249,7 +3253,6 @@
     <mergeCell ref="E25:M25"/>
     <mergeCell ref="E21:M21"/>
     <mergeCell ref="E22:M22"/>
-    <mergeCell ref="B36:D36"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="E35:M35"/>
     <mergeCell ref="E36:M36"/>
@@ -3368,24 +3371,24 @@
     <mergeCell ref="B62:C62"/>
     <mergeCell ref="D62:E62"/>
   </mergeCells>
-  <conditionalFormatting sqref="A77:D77 K77:M77 C79:J79 D51:J55 D50:E50 H50:J50 D48:J49">
-    <cfRule type="containsBlanks" dxfId="5" priority="2">
-      <formula>LEN(TRIM(A48))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A77:D77">
-    <cfRule type="containsBlanks" dxfId="4" priority="4">
+    <cfRule type="containsBlanks" dxfId="5" priority="4">
       <formula>LEN(TRIM(A77))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C79">
-    <cfRule type="containsBlanks" dxfId="3" priority="5">
+    <cfRule type="containsBlanks" dxfId="4" priority="5">
       <formula>LEN(TRIM(C79))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D42:F43 J42:J43 D59:J63 B68:J68 B70:J70">
-    <cfRule type="containsBlanks" dxfId="2" priority="1">
+    <cfRule type="containsBlanks" dxfId="3" priority="1">
       <formula>LEN(TRIM(B42))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A77:D77 K77:M77 C79:J79 D48:J55">
+    <cfRule type="containsBlanks" dxfId="2" priority="2">
+      <formula>LEN(TRIM(A48))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:M10 C11:H11 K11:M11 J13:M13 E14:M22 E26:M37">
@@ -3445,7 +3448,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OBLIGATORIO" prompt="Registrar de manera objetiva y concisa la información adicional que complemente el proceso de acompañamiento al aprendiz en su etapa productiva." sqref="B70:J70 B68:J68" xr:uid="{D7E55FAF-6FC8-4AC1-A902-F35811C9DD3B}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="DILIGENCIAR SI HAY POR MEJORAR" prompt="Si hay factores por mejorar favor escribir las observaciones o los compromisos de mejora" sqref="H48:J55" xr:uid="{70C7BBAF-F2BE-4776-BA55-57FE0807C14D}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Diligenciar si hay por mejorar" prompt="Si hay factores por mejorar favor escribir las observaciones o los compromisos de mejora" sqref="H59:J63" xr:uid="{56231F2E-9BAE-4742-84BB-A6BBFCFB029F}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Realiza acciones que fortalezcan su perfil ocupacional potenciando sus competencias en el marco de su proyecto de vida." sqref="D50:E50 F49:G49" xr:uid="{379961D4-6BD4-47A0-B009-E49C8B35A883}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Realiza acciones que fortalezcan su perfil ocupacional potenciando sus competencias en el marco de su proyecto de vida." sqref="D50:G50 F49:G49" xr:uid="{379961D4-6BD4-47A0-B009-E49C8B35A883}"/>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" scale="68" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>